<commit_message>
Regenerar CSV, Excel y PNG con KPIs actualizados en el README.
Salidas coherentes con el nuevo flujo de caja y la convención ARS (USD).

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/excel/dashboard_costos.xlsx
+++ b/excel/dashboard_costos.xlsx
@@ -21,8 +21,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
-    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="#.##0,00 &quot;ARS&quot;"/>
+    <numFmt numFmtId="165" formatCode="#.##0,00 &quot;USD&quot;"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -935,36 +935,36 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Costo total último mes (ARS)</t>
+          <t>Costo total último mes</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>$93,186,309</t>
+          <t>ARS 81,4 M (USD 53,7 k)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Costos fijos (ARS)</t>
+          <t>Costos fijos</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>$27,060,000</t>
+          <t>ARS 27,1 M (USD 17,9 k)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Costos variables (ARS)</t>
+          <t>Costos variables</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>$66,126,309</t>
+          <t>ARS 54,3 M (USD 35,9 k)</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>25,703</t>
+          <t>25.312</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>1.62%</t>
+          <t>-1,28%</t>
         </is>
       </c>
     </row>
@@ -1078,23 +1078,23 @@
       <c r="C2" s="7" t="n">
         <v>22000000</v>
       </c>
-      <c r="D2" s="6" t="n">
+      <c r="D2" s="8" t="n">
         <v>14525.62</v>
       </c>
       <c r="E2" s="7" t="n">
-        <v>43980075.06</v>
-      </c>
-      <c r="F2" s="6" t="n">
-        <v>29038.08</v>
+        <v>45447172.45</v>
+      </c>
+      <c r="F2" s="8" t="n">
+        <v>30006.74</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>65980075.06</v>
-      </c>
-      <c r="H2" s="6" t="n">
-        <v>43563.7</v>
+        <v>67447172.45</v>
+      </c>
+      <c r="H2" s="8" t="n">
+        <v>44532.36</v>
       </c>
       <c r="I2" s="6" t="n">
-        <v>18402</v>
+        <v>17987</v>
       </c>
     </row>
     <row r="3">
@@ -1111,23 +1111,23 @@
       <c r="C3" s="7" t="n">
         <v>22220000</v>
       </c>
-      <c r="D3" s="6" t="n">
+      <c r="D3" s="8" t="n">
         <v>14670.87</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>42119825.81</v>
-      </c>
-      <c r="F3" s="6" t="n">
-        <v>27809.84</v>
+        <v>47179459.18</v>
+      </c>
+      <c r="F3" s="8" t="n">
+        <v>31150.49</v>
       </c>
       <c r="G3" s="7" t="n">
-        <v>64339825.81</v>
-      </c>
-      <c r="H3" s="6" t="n">
-        <v>42480.72</v>
+        <v>69399459.18000001</v>
+      </c>
+      <c r="H3" s="8" t="n">
+        <v>45821.37</v>
       </c>
       <c r="I3" s="6" t="n">
-        <v>18978</v>
+        <v>18954</v>
       </c>
     </row>
     <row r="4">
@@ -1144,23 +1144,23 @@
       <c r="C4" s="7" t="n">
         <v>22440000</v>
       </c>
-      <c r="D4" s="6" t="n">
+      <c r="D4" s="8" t="n">
         <v>14816.13</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>49826518.45</v>
-      </c>
-      <c r="F4" s="6" t="n">
-        <v>32898.23</v>
+        <v>44084639.24</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>29107.12</v>
       </c>
       <c r="G4" s="7" t="n">
-        <v>72266518.45</v>
-      </c>
-      <c r="H4" s="6" t="n">
-        <v>47714.36</v>
+        <v>66524639.24</v>
+      </c>
+      <c r="H4" s="8" t="n">
+        <v>43923.25</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>19235</v>
+        <v>18289</v>
       </c>
     </row>
     <row r="5">
@@ -1177,23 +1177,23 @@
       <c r="C5" s="7" t="n">
         <v>22660000</v>
       </c>
-      <c r="D5" s="6" t="n">
+      <c r="D5" s="8" t="n">
         <v>14961.39</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>42852921.1</v>
-      </c>
-      <c r="F5" s="6" t="n">
-        <v>28293.87</v>
+        <v>44361321.46</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>29289.8</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>65512921.1</v>
-      </c>
-      <c r="H5" s="6" t="n">
-        <v>43255.26</v>
+        <v>67021321.46</v>
+      </c>
+      <c r="H5" s="8" t="n">
+        <v>44251.19</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>19729</v>
+        <v>19436</v>
       </c>
     </row>
     <row r="6">
@@ -1210,23 +1210,23 @@
       <c r="C6" s="7" t="n">
         <v>22880000</v>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="D6" s="8" t="n">
         <v>15106.64</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>50545358.09</v>
-      </c>
-      <c r="F6" s="6" t="n">
-        <v>33372.84</v>
+        <v>48186897.22</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>31815.66</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>73425358.09</v>
-      </c>
-      <c r="H6" s="6" t="n">
-        <v>48479.49</v>
+        <v>71066897.22</v>
+      </c>
+      <c r="H6" s="8" t="n">
+        <v>46922.3</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>19981</v>
+        <v>19158</v>
       </c>
     </row>
     <row r="7">
@@ -1243,23 +1243,23 @@
       <c r="C7" s="7" t="n">
         <v>23100000</v>
       </c>
-      <c r="D7" s="6" t="n">
+      <c r="D7" s="8" t="n">
         <v>15251.9</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>48020734.51</v>
-      </c>
-      <c r="F7" s="6" t="n">
-        <v>31705.95</v>
+        <v>49113724.63</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>32427.6</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>71120734.51000001</v>
-      </c>
-      <c r="H7" s="6" t="n">
-        <v>46957.85</v>
+        <v>72213724.63</v>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>47679.5</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>19415</v>
+        <v>19412</v>
       </c>
     </row>
     <row r="8">
@@ -1276,23 +1276,23 @@
       <c r="C8" s="7" t="n">
         <v>23320000</v>
       </c>
-      <c r="D8" s="6" t="n">
+      <c r="D8" s="8" t="n">
         <v>15397.16</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>45356710.26</v>
-      </c>
-      <c r="F8" s="6" t="n">
-        <v>29947.01</v>
+        <v>51165356.46</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>33782.2</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>68676710.26000001</v>
-      </c>
-      <c r="H8" s="6" t="n">
-        <v>45344.17</v>
+        <v>74485356.45999999</v>
+      </c>
+      <c r="H8" s="8" t="n">
+        <v>49179.36</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>19900</v>
+        <v>20677</v>
       </c>
     </row>
     <row r="9">
@@ -1309,23 +1309,23 @@
       <c r="C9" s="7" t="n">
         <v>23540000</v>
       </c>
-      <c r="D9" s="6" t="n">
+      <c r="D9" s="8" t="n">
         <v>15542.41</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>52838531.47</v>
-      </c>
-      <c r="F9" s="6" t="n">
-        <v>34886.92</v>
+        <v>46201076.56</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>30504.51</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>76378531.47</v>
-      </c>
-      <c r="H9" s="6" t="n">
-        <v>50429.34</v>
+        <v>69741076.56</v>
+      </c>
+      <c r="H9" s="8" t="n">
+        <v>46046.92</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>20669</v>
+        <v>20899</v>
       </c>
     </row>
     <row r="10">
@@ -1342,23 +1342,23 @@
       <c r="C10" s="7" t="n">
         <v>23760000</v>
       </c>
-      <c r="D10" s="6" t="n">
+      <c r="D10" s="8" t="n">
         <v>15687.67</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>53778002.86</v>
-      </c>
-      <c r="F10" s="6" t="n">
-        <v>35507.22</v>
+        <v>44789262.93</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>29572.35</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>77538002.86</v>
-      </c>
-      <c r="H10" s="6" t="n">
-        <v>51194.88</v>
+        <v>68549262.93000001</v>
+      </c>
+      <c r="H10" s="8" t="n">
+        <v>45260.02</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>20904</v>
+        <v>20199</v>
       </c>
     </row>
     <row r="11">
@@ -1375,23 +1375,23 @@
       <c r="C11" s="7" t="n">
         <v>23980000</v>
       </c>
-      <c r="D11" s="6" t="n">
+      <c r="D11" s="8" t="n">
         <v>15832.92</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>50417749.21</v>
-      </c>
-      <c r="F11" s="6" t="n">
-        <v>33288.59</v>
+        <v>46625039.14</v>
+      </c>
+      <c r="F11" s="8" t="n">
+        <v>30784.43</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>74397749.20999999</v>
-      </c>
-      <c r="H11" s="6" t="n">
-        <v>49121.51</v>
+        <v>70605039.14</v>
+      </c>
+      <c r="H11" s="8" t="n">
+        <v>46617.36</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>21131</v>
+        <v>21691</v>
       </c>
     </row>
     <row r="12">
@@ -1408,23 +1408,23 @@
       <c r="C12" s="7" t="n">
         <v>24200000</v>
       </c>
-      <c r="D12" s="6" t="n">
+      <c r="D12" s="8" t="n">
         <v>15978.18</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>53150416.32</v>
-      </c>
-      <c r="F12" s="6" t="n">
-        <v>35092.85</v>
+        <v>50478185.96</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>33328.49</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>77350416.31999999</v>
-      </c>
-      <c r="H12" s="6" t="n">
-        <v>51071.03</v>
+        <v>74678185.95999999</v>
+      </c>
+      <c r="H12" s="8" t="n">
+        <v>49306.67</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>20800</v>
+        <v>22104</v>
       </c>
     </row>
     <row r="13">
@@ -1441,23 +1441,23 @@
       <c r="C13" s="7" t="n">
         <v>24420000</v>
       </c>
-      <c r="D13" s="6" t="n">
+      <c r="D13" s="8" t="n">
         <v>16123.44</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>55599109.26</v>
-      </c>
-      <c r="F13" s="6" t="n">
-        <v>36709.61</v>
+        <v>53629693.25</v>
+      </c>
+      <c r="F13" s="8" t="n">
+        <v>35409.29</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>80019109.26000001</v>
-      </c>
-      <c r="H13" s="6" t="n">
-        <v>52833.05</v>
+        <v>78049693.25</v>
+      </c>
+      <c r="H13" s="8" t="n">
+        <v>51532.73</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>22597</v>
+        <v>22359</v>
       </c>
     </row>
     <row r="14">
@@ -1474,23 +1474,23 @@
       <c r="C14" s="7" t="n">
         <v>24640000</v>
       </c>
-      <c r="D14" s="6" t="n">
+      <c r="D14" s="8" t="n">
         <v>16268.69</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>55143103.35</v>
-      </c>
-      <c r="F14" s="6" t="n">
-        <v>36408.53</v>
+        <v>49535648.68</v>
+      </c>
+      <c r="F14" s="8" t="n">
+        <v>32706.18</v>
       </c>
       <c r="G14" s="7" t="n">
-        <v>79783103.34999999</v>
-      </c>
-      <c r="H14" s="6" t="n">
-        <v>52677.22</v>
+        <v>74175648.68000001</v>
+      </c>
+      <c r="H14" s="8" t="n">
+        <v>48974.87</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>21584</v>
+        <v>21877</v>
       </c>
     </row>
     <row r="15">
@@ -1507,23 +1507,23 @@
       <c r="C15" s="7" t="n">
         <v>24860000</v>
       </c>
-      <c r="D15" s="6" t="n">
+      <c r="D15" s="8" t="n">
         <v>16413.95</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>58742822.18</v>
-      </c>
-      <c r="F15" s="6" t="n">
-        <v>38785.26</v>
+        <v>47220987.01</v>
+      </c>
+      <c r="F15" s="8" t="n">
+        <v>31177.91</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>83602822.18000001</v>
-      </c>
-      <c r="H15" s="6" t="n">
-        <v>55199.21</v>
+        <v>72080987.01000001</v>
+      </c>
+      <c r="H15" s="8" t="n">
+        <v>47591.86</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>22736</v>
+        <v>21802</v>
       </c>
     </row>
     <row r="16">
@@ -1540,23 +1540,23 @@
       <c r="C16" s="7" t="n">
         <v>25080000</v>
       </c>
-      <c r="D16" s="6" t="n">
+      <c r="D16" s="8" t="n">
         <v>16559.2</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>59198825.86</v>
-      </c>
-      <c r="F16" s="6" t="n">
-        <v>39086.34</v>
+        <v>57291998.11</v>
+      </c>
+      <c r="F16" s="8" t="n">
+        <v>37827.35</v>
       </c>
       <c r="G16" s="7" t="n">
-        <v>84278825.86</v>
-      </c>
-      <c r="H16" s="6" t="n">
-        <v>55645.55</v>
+        <v>82371998.11</v>
+      </c>
+      <c r="H16" s="8" t="n">
+        <v>54386.55</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>22913</v>
+        <v>23018</v>
       </c>
     </row>
     <row r="17">
@@ -1573,23 +1573,23 @@
       <c r="C17" s="7" t="n">
         <v>25300000</v>
       </c>
-      <c r="D17" s="6" t="n">
+      <c r="D17" s="8" t="n">
         <v>16704.46</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>61058957.24</v>
-      </c>
-      <c r="F17" s="6" t="n">
-        <v>40314.5</v>
+        <v>47961981.2</v>
+      </c>
+      <c r="F17" s="8" t="n">
+        <v>31667.16</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>86358957.23999999</v>
-      </c>
-      <c r="H17" s="6" t="n">
-        <v>57018.97</v>
+        <v>73261981.2</v>
+      </c>
+      <c r="H17" s="8" t="n">
+        <v>48371.62</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>23757</v>
+        <v>22513</v>
       </c>
     </row>
     <row r="18">
@@ -1606,23 +1606,23 @@
       <c r="C18" s="7" t="n">
         <v>25520000</v>
       </c>
-      <c r="D18" s="6" t="n">
+      <c r="D18" s="8" t="n">
         <v>16849.72</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>54555289.44</v>
-      </c>
-      <c r="F18" s="6" t="n">
-        <v>36020.42</v>
+        <v>56355264.81</v>
+      </c>
+      <c r="F18" s="8" t="n">
+        <v>37208.87</v>
       </c>
       <c r="G18" s="7" t="n">
-        <v>80075289.44</v>
-      </c>
-      <c r="H18" s="6" t="n">
-        <v>52870.14</v>
+        <v>81875264.81</v>
+      </c>
+      <c r="H18" s="8" t="n">
+        <v>54058.58</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>24235</v>
+        <v>23363</v>
       </c>
     </row>
     <row r="19">
@@ -1639,23 +1639,23 @@
       <c r="C19" s="7" t="n">
         <v>25740000</v>
       </c>
-      <c r="D19" s="6" t="n">
+      <c r="D19" s="8" t="n">
         <v>16994.97</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>63139132.29</v>
-      </c>
-      <c r="F19" s="6" t="n">
-        <v>41687.95</v>
+        <v>59399474.56</v>
+      </c>
+      <c r="F19" s="8" t="n">
+        <v>39218.82</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>88879132.29000001</v>
-      </c>
-      <c r="H19" s="6" t="n">
-        <v>58682.92</v>
+        <v>85139474.56</v>
+      </c>
+      <c r="H19" s="8" t="n">
+        <v>56213.8</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>24523</v>
+        <v>24490</v>
       </c>
     </row>
     <row r="20">
@@ -1672,23 +1672,23 @@
       <c r="C20" s="7" t="n">
         <v>25960000</v>
       </c>
-      <c r="D20" s="6" t="n">
+      <c r="D20" s="8" t="n">
         <v>17140.23</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>50944973.23</v>
-      </c>
-      <c r="F20" s="6" t="n">
-        <v>33636.69</v>
+        <v>54994124.76</v>
+      </c>
+      <c r="F20" s="8" t="n">
+        <v>36310.17</v>
       </c>
       <c r="G20" s="7" t="n">
-        <v>76904973.23</v>
-      </c>
-      <c r="H20" s="6" t="n">
-        <v>50776.92</v>
+        <v>80954124.76000001</v>
+      </c>
+      <c r="H20" s="8" t="n">
+        <v>53450.4</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>24072</v>
+        <v>24374</v>
       </c>
     </row>
     <row r="21">
@@ -1705,23 +1705,23 @@
       <c r="C21" s="7" t="n">
         <v>26180000</v>
       </c>
-      <c r="D21" s="6" t="n">
+      <c r="D21" s="8" t="n">
         <v>17285.49</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>55198807.87</v>
-      </c>
-      <c r="F21" s="6" t="n">
-        <v>36445.31</v>
+        <v>57352318.33</v>
+      </c>
+      <c r="F21" s="8" t="n">
+        <v>37867.18</v>
       </c>
       <c r="G21" s="7" t="n">
-        <v>81378807.87</v>
-      </c>
-      <c r="H21" s="6" t="n">
-        <v>53730.79</v>
+        <v>83532318.33</v>
+      </c>
+      <c r="H21" s="8" t="n">
+        <v>55152.66</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>24665</v>
+        <v>24116</v>
       </c>
     </row>
     <row r="22">
@@ -1738,23 +1738,23 @@
       <c r="C22" s="7" t="n">
         <v>26400000</v>
       </c>
-      <c r="D22" s="6" t="n">
+      <c r="D22" s="8" t="n">
         <v>17430.74</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>60983261.7</v>
-      </c>
-      <c r="F22" s="6" t="n">
-        <v>40264.53</v>
+        <v>59498682.88</v>
+      </c>
+      <c r="F22" s="8" t="n">
+        <v>39284.32</v>
       </c>
       <c r="G22" s="7" t="n">
-        <v>87383261.7</v>
-      </c>
-      <c r="H22" s="6" t="n">
-        <v>57695.27</v>
+        <v>85898682.88</v>
+      </c>
+      <c r="H22" s="8" t="n">
+        <v>56715.07</v>
       </c>
       <c r="I22" s="6" t="n">
-        <v>24457</v>
+        <v>24789</v>
       </c>
     </row>
     <row r="23">
@@ -1771,23 +1771,23 @@
       <c r="C23" s="7" t="n">
         <v>26620000</v>
       </c>
-      <c r="D23" s="6" t="n">
+      <c r="D23" s="8" t="n">
         <v>17576</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>63525993.34</v>
-      </c>
-      <c r="F23" s="6" t="n">
-        <v>41943.38</v>
+        <v>56931471.35</v>
+      </c>
+      <c r="F23" s="8" t="n">
+        <v>37589.31</v>
       </c>
       <c r="G23" s="7" t="n">
-        <v>90145993.34</v>
-      </c>
-      <c r="H23" s="6" t="n">
-        <v>59519.38</v>
+        <v>83551471.34999999</v>
+      </c>
+      <c r="H23" s="8" t="n">
+        <v>55165.31</v>
       </c>
       <c r="I23" s="6" t="n">
-        <v>25117</v>
+        <v>25725</v>
       </c>
     </row>
     <row r="24">
@@ -1804,23 +1804,23 @@
       <c r="C24" s="7" t="n">
         <v>26840000</v>
       </c>
-      <c r="D24" s="6" t="n">
+      <c r="D24" s="8" t="n">
         <v>17721.25</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>53884005.92</v>
-      </c>
-      <c r="F24" s="6" t="n">
-        <v>35577.2</v>
+        <v>54665402.37</v>
+      </c>
+      <c r="F24" s="8" t="n">
+        <v>36093.13</v>
       </c>
       <c r="G24" s="7" t="n">
-        <v>80724005.92</v>
-      </c>
-      <c r="H24" s="6" t="n">
-        <v>53298.46</v>
+        <v>81505402.37</v>
+      </c>
+      <c r="H24" s="8" t="n">
+        <v>53814.38</v>
       </c>
       <c r="I24" s="6" t="n">
-        <v>25563</v>
+        <v>24959</v>
       </c>
     </row>
     <row r="25">
@@ -1837,23 +1837,23 @@
       <c r="C25" s="7" t="n">
         <v>27060000</v>
       </c>
-      <c r="D25" s="6" t="n">
+      <c r="D25" s="8" t="n">
         <v>17866.51</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>66126309.14</v>
-      </c>
-      <c r="F25" s="6" t="n">
-        <v>43660.25</v>
+        <v>54316485.24</v>
+      </c>
+      <c r="F25" s="8" t="n">
+        <v>35862.75</v>
       </c>
       <c r="G25" s="7" t="n">
-        <v>93186309.14</v>
-      </c>
-      <c r="H25" s="6" t="n">
-        <v>61526.76</v>
+        <v>81376485.23999999</v>
+      </c>
+      <c r="H25" s="8" t="n">
+        <v>53729.26</v>
       </c>
       <c r="I25" s="6" t="n">
-        <v>25703</v>
+        <v>25312</v>
       </c>
     </row>
   </sheetData>
@@ -1925,10 +1925,10 @@
         </is>
       </c>
       <c r="E2" s="7" t="n">
-        <v>37351060.51</v>
-      </c>
-      <c r="F2" s="6" t="n">
-        <v>24661.24</v>
+        <v>34282307.91</v>
+      </c>
+      <c r="F2" s="8" t="n">
+        <v>22635.08</v>
       </c>
     </row>
     <row r="3">
@@ -1953,10 +1953,10 @@
         </is>
       </c>
       <c r="E3" s="7" t="n">
-        <v>26831167.15</v>
-      </c>
-      <c r="F3" s="6" t="n">
-        <v>17715.42</v>
+        <v>22503319.67</v>
+      </c>
+      <c r="F3" s="8" t="n">
+        <v>14857.94</v>
       </c>
     </row>
     <row r="4">
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E4" s="7" t="n">
-        <v>17389092.38</v>
-      </c>
-      <c r="F4" s="6" t="n">
-        <v>11481.24</v>
+        <v>14579868.78</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>9626.440000000001</v>
       </c>
     </row>
     <row r="5">
@@ -2009,10 +2009,10 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>11206344.61</v>
-      </c>
-      <c r="F5" s="6" t="n">
-        <v>7399.05</v>
+        <v>9430632.279999999</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>6226.63</v>
       </c>
     </row>
   </sheetData>
@@ -2088,14 +2088,14 @@
           <t>Yerba mate premium 1kg</t>
         </is>
       </c>
-      <c r="E2" s="8" t="n">
-        <v>1553.69</v>
+      <c r="E2" s="7" t="n">
+        <v>1397.68</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>1.03</v>
+        <v>0.92</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>6425</v>
+        <v>6328</v>
       </c>
     </row>
     <row r="3">
@@ -2119,14 +2119,14 @@
           <t>Aceite de girasol 900ml</t>
         </is>
       </c>
-      <c r="E3" s="8" t="n">
-        <v>2092.87</v>
+      <c r="E3" s="7" t="n">
+        <v>1411.26</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>1.38</v>
+        <v>0.93</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>6425</v>
+        <v>6328</v>
       </c>
     </row>
     <row r="4">
@@ -2150,14 +2150,14 @@
           <t>Arroz largo fino 1kg</t>
         </is>
       </c>
-      <c r="E4" s="8" t="n">
-        <v>1130.42</v>
+      <c r="E4" s="7" t="n">
+        <v>2068.76</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>0.75</v>
+        <v>1.37</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>6425</v>
+        <v>6328</v>
       </c>
     </row>
     <row r="5">
@@ -2181,14 +2181,14 @@
           <t>Harina 000 1kg</t>
         </is>
       </c>
-      <c r="E5" s="8" t="n">
-        <v>1576</v>
+      <c r="E5" s="7" t="n">
+        <v>1700.94</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>1.04</v>
+        <v>1.12</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>6425</v>
+        <v>6328</v>
       </c>
     </row>
   </sheetData>
@@ -2260,22 +2260,22 @@
         </is>
       </c>
       <c r="C2" s="7" t="n">
-        <v>66783455.11</v>
-      </c>
-      <c r="D2" s="6" t="n">
-        <v>44094.13</v>
+        <v>64782056.64</v>
+      </c>
+      <c r="D2" s="8" t="n">
+        <v>42772.7</v>
       </c>
       <c r="E2" s="7" t="n">
-        <v>65980075.06</v>
-      </c>
-      <c r="F2" s="6" t="n">
-        <v>43563.7</v>
+        <v>67447172.45</v>
+      </c>
+      <c r="F2" s="8" t="n">
+        <v>44532.36</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>-803380.0600000001</v>
+        <v>2665115.8</v>
       </c>
       <c r="H2" s="6" t="n">
-        <v>-1.2</v>
+        <v>4.11</v>
       </c>
     </row>
     <row r="3">
@@ -2290,22 +2290,22 @@
         </is>
       </c>
       <c r="C3" s="7" t="n">
-        <v>64825180.98</v>
-      </c>
-      <c r="D3" s="6" t="n">
-        <v>42801.17</v>
+        <v>67535408.61</v>
+      </c>
+      <c r="D3" s="8" t="n">
+        <v>44590.62</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>64339825.81</v>
-      </c>
-      <c r="F3" s="6" t="n">
-        <v>42480.72</v>
+        <v>69399459.18000001</v>
+      </c>
+      <c r="F3" s="8" t="n">
+        <v>45821.37</v>
       </c>
       <c r="G3" s="7" t="n">
-        <v>-485355.17</v>
+        <v>1864050.57</v>
       </c>
       <c r="H3" s="6" t="n">
-        <v>-0.75</v>
+        <v>2.76</v>
       </c>
     </row>
     <row r="4">
@@ -2320,22 +2320,22 @@
         </is>
       </c>
       <c r="C4" s="7" t="n">
-        <v>71357093.78</v>
-      </c>
-      <c r="D4" s="6" t="n">
-        <v>47113.9</v>
+        <v>65623189.89</v>
+      </c>
+      <c r="D4" s="8" t="n">
+        <v>43328.06</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>72266518.45</v>
-      </c>
-      <c r="F4" s="6" t="n">
-        <v>47714.36</v>
+        <v>66524639.24</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>43923.25</v>
       </c>
       <c r="G4" s="7" t="n">
-        <v>909424.67</v>
+        <v>901449.35</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>1.27</v>
+        <v>1.37</v>
       </c>
     </row>
     <row r="5">
@@ -2350,22 +2350,22 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>64183921.75</v>
-      </c>
-      <c r="D5" s="6" t="n">
-        <v>42377.78</v>
+        <v>66358325.49</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>43813.44</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>65512921.1</v>
-      </c>
-      <c r="F5" s="6" t="n">
-        <v>43255.26</v>
+        <v>67021321.46</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>44251.19</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>1328999.35</v>
+        <v>662995.97</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>2.07</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -2380,22 +2380,22 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>74545516.7</v>
-      </c>
-      <c r="D6" s="6" t="n">
-        <v>49219.08</v>
+        <v>68824411.19</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>45441.69</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>73425358.09</v>
-      </c>
-      <c r="F6" s="6" t="n">
-        <v>48479.49</v>
+        <v>71066897.22</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>46922.3</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>-1120158.61</v>
+        <v>2242486.03</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>-1.5</v>
+        <v>3.26</v>
       </c>
     </row>
     <row r="7">
@@ -2410,22 +2410,22 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>71673243.61</v>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>47322.64</v>
+        <v>71295683.23</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>47073.36</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>71120734.51000001</v>
-      </c>
-      <c r="F7" s="6" t="n">
-        <v>46957.85</v>
+        <v>72213724.63</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>47679.5</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>-552509.1</v>
+        <v>918041.41</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>-0.77</v>
+        <v>1.29</v>
       </c>
     </row>
     <row r="8">
@@ -2440,22 +2440,22 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>68744567.98</v>
-      </c>
-      <c r="D8" s="6" t="n">
-        <v>45388.97</v>
+        <v>72971842.09</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>48180.05</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>68676710.26000001</v>
-      </c>
-      <c r="F8" s="6" t="n">
-        <v>45344.17</v>
+        <v>74485356.45999999</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>49179.36</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>-67857.73</v>
+        <v>1513514.37</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>-0.1</v>
+        <v>2.07</v>
       </c>
     </row>
     <row r="9">
@@ -2470,22 +2470,22 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>74047346.97</v>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>48890.16</v>
+        <v>69012803.77</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>45566.07</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>76378531.47</v>
-      </c>
-      <c r="F9" s="6" t="n">
-        <v>50429.34</v>
+        <v>69741076.56</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>46046.92</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>2331184.5</v>
+        <v>728272.79</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>3.15</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="10">
@@ -2500,22 +2500,22 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>74932663.62</v>
-      </c>
-      <c r="D10" s="6" t="n">
-        <v>49474.69</v>
+        <v>69448960.15000001</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>45854.05</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>77538002.86</v>
-      </c>
-      <c r="F10" s="6" t="n">
-        <v>51194.88</v>
+        <v>68549262.93000001</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>45260.02</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>2605339.23</v>
+        <v>-899697.22</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>3.48</v>
+        <v>-1.3</v>
       </c>
     </row>
     <row r="11">
@@ -2530,22 +2530,22 @@
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>74745940.38</v>
-      </c>
-      <c r="D11" s="6" t="n">
-        <v>49351.41</v>
+        <v>68201733.8</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>45030.56</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>74397749.20999999</v>
-      </c>
-      <c r="F11" s="6" t="n">
-        <v>49121.51</v>
+        <v>70605039.14</v>
+      </c>
+      <c r="F11" s="8" t="n">
+        <v>46617.36</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>-348191.17</v>
+        <v>2403305.34</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>-0.47</v>
+        <v>3.52</v>
       </c>
     </row>
     <row r="12">
@@ -2560,22 +2560,22 @@
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>75419564.91</v>
-      </c>
-      <c r="D12" s="6" t="n">
-        <v>49796.17</v>
+        <v>72641439.17</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>47961.9</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>77350416.31999999</v>
-      </c>
-      <c r="F12" s="6" t="n">
-        <v>51071.03</v>
+        <v>74678185.95999999</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>49306.67</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>1930851.41</v>
+        <v>2036746.79</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>2.56</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="13">
@@ -2590,22 +2590,22 @@
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>80334511.47</v>
-      </c>
-      <c r="D13" s="6" t="n">
-        <v>53041.29</v>
+        <v>75939001.73</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>50139.13</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>80019109.26000001</v>
-      </c>
-      <c r="F13" s="6" t="n">
-        <v>52833.05</v>
+        <v>78049693.25</v>
+      </c>
+      <c r="F13" s="8" t="n">
+        <v>51532.73</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>-315402.21</v>
+        <v>2110691.52</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>-0.39</v>
+        <v>2.78</v>
       </c>
     </row>
     <row r="14">
@@ -2620,22 +2620,22 @@
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>77379451.09</v>
-      </c>
-      <c r="D14" s="6" t="n">
-        <v>51090.2</v>
+        <v>74150685.5</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>48958.39</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>79783103.34999999</v>
-      </c>
-      <c r="F14" s="6" t="n">
-        <v>52677.22</v>
+        <v>74175648.68000001</v>
+      </c>
+      <c r="F14" s="8" t="n">
+        <v>48974.87</v>
       </c>
       <c r="G14" s="7" t="n">
-        <v>2403652.26</v>
+        <v>24963.18</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>3.11</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="15">
@@ -2650,22 +2650,22 @@
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>83641645.14</v>
-      </c>
-      <c r="D15" s="6" t="n">
-        <v>55224.85</v>
+        <v>69472627.09</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>45869.67</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>83602822.18000001</v>
-      </c>
-      <c r="F15" s="6" t="n">
-        <v>55199.21</v>
+        <v>72080987.01000001</v>
+      </c>
+      <c r="F15" s="8" t="n">
+        <v>47591.86</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>-38822.96</v>
+        <v>2608359.91</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>-0.05</v>
+        <v>3.75</v>
       </c>
     </row>
     <row r="16">
@@ -2680,22 +2680,22 @@
         </is>
       </c>
       <c r="C16" s="7" t="n">
-        <v>83863635.12</v>
-      </c>
-      <c r="D16" s="6" t="n">
-        <v>55371.42</v>
+        <v>81340910.84999999</v>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>53705.77</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>84278825.86</v>
-      </c>
-      <c r="F16" s="6" t="n">
-        <v>55645.55</v>
+        <v>82371998.11</v>
+      </c>
+      <c r="F16" s="8" t="n">
+        <v>54386.55</v>
       </c>
       <c r="G16" s="7" t="n">
-        <v>415190.74</v>
+        <v>1031087.26</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>0.5</v>
+        <v>1.27</v>
       </c>
     </row>
     <row r="17">
@@ -2710,22 +2710,22 @@
         </is>
       </c>
       <c r="C17" s="7" t="n">
-        <v>87173436.29000001</v>
-      </c>
-      <c r="D17" s="6" t="n">
-        <v>57556.73</v>
+        <v>70620222.58</v>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>46627.38</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>86358957.23999999</v>
-      </c>
-      <c r="F17" s="6" t="n">
-        <v>57018.97</v>
+        <v>73261981.2</v>
+      </c>
+      <c r="F17" s="8" t="n">
+        <v>48371.62</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>-814479.05</v>
+        <v>2641758.62</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>-0.93</v>
+        <v>3.74</v>
       </c>
     </row>
     <row r="18">
@@ -2740,22 +2740,22 @@
         </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>79051817.17</v>
-      </c>
-      <c r="D18" s="6" t="n">
-        <v>52194.39</v>
+        <v>79162315.17</v>
+      </c>
+      <c r="D18" s="8" t="n">
+        <v>52267.34</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>80075289.44</v>
-      </c>
-      <c r="F18" s="6" t="n">
-        <v>52870.14</v>
+        <v>81875264.81</v>
+      </c>
+      <c r="F18" s="8" t="n">
+        <v>54058.58</v>
       </c>
       <c r="G18" s="7" t="n">
-        <v>1023472.27</v>
+        <v>2712949.64</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>1.29</v>
+        <v>3.43</v>
       </c>
     </row>
     <row r="19">
@@ -2770,22 +2770,22 @@
         </is>
       </c>
       <c r="C19" s="7" t="n">
-        <v>90331700.3</v>
-      </c>
-      <c r="D19" s="6" t="n">
-        <v>59641.99</v>
+        <v>82219629.08</v>
+      </c>
+      <c r="D19" s="8" t="n">
+        <v>54285.95</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>88879132.29000001</v>
-      </c>
-      <c r="F19" s="6" t="n">
-        <v>58682.92</v>
+        <v>85139474.56</v>
+      </c>
+      <c r="F19" s="8" t="n">
+        <v>56213.8</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>-1452568.01</v>
+        <v>2919845.48</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>-1.61</v>
+        <v>3.55</v>
       </c>
     </row>
     <row r="20">
@@ -2800,22 +2800,22 @@
         </is>
       </c>
       <c r="C20" s="7" t="n">
-        <v>75483802.43000001</v>
-      </c>
-      <c r="D20" s="6" t="n">
-        <v>49838.59</v>
+        <v>79525997.79000001</v>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>52507.47</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>76904973.23</v>
-      </c>
-      <c r="F20" s="6" t="n">
-        <v>50776.92</v>
+        <v>80954124.76000001</v>
+      </c>
+      <c r="F20" s="8" t="n">
+        <v>53450.4</v>
       </c>
       <c r="G20" s="7" t="n">
-        <v>1421170.8</v>
+        <v>1428126.97</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>1.88</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="21">
@@ -2830,22 +2830,22 @@
         </is>
       </c>
       <c r="C21" s="7" t="n">
-        <v>79752090.20999999</v>
-      </c>
-      <c r="D21" s="6" t="n">
-        <v>52656.75</v>
+        <v>83804937.81</v>
+      </c>
+      <c r="D21" s="8" t="n">
+        <v>55332.66</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>81378807.87</v>
-      </c>
-      <c r="F21" s="6" t="n">
-        <v>53730.79</v>
+        <v>83532318.33</v>
+      </c>
+      <c r="F21" s="8" t="n">
+        <v>55152.66</v>
       </c>
       <c r="G21" s="7" t="n">
-        <v>1626717.66</v>
+        <v>-272619.48</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>2.04</v>
+        <v>-0.33</v>
       </c>
     </row>
     <row r="22">
@@ -2860,22 +2860,22 @@
         </is>
       </c>
       <c r="C22" s="7" t="n">
-        <v>87012660.38</v>
-      </c>
-      <c r="D22" s="6" t="n">
-        <v>57450.58</v>
+        <v>86393144.72</v>
+      </c>
+      <c r="D22" s="8" t="n">
+        <v>57041.54</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>87383261.7</v>
-      </c>
-      <c r="F22" s="6" t="n">
-        <v>57695.27</v>
+        <v>85898682.88</v>
+      </c>
+      <c r="F22" s="8" t="n">
+        <v>56715.07</v>
       </c>
       <c r="G22" s="7" t="n">
-        <v>370601.32</v>
+        <v>-494461.85</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>0.43</v>
+        <v>-0.57</v>
       </c>
     </row>
     <row r="23">
@@ -2890,22 +2890,22 @@
         </is>
       </c>
       <c r="C23" s="7" t="n">
-        <v>87827068.45999999</v>
-      </c>
-      <c r="D23" s="6" t="n">
-        <v>57988.29</v>
+        <v>83685844.78</v>
+      </c>
+      <c r="D23" s="8" t="n">
+        <v>55254.03</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>90145993.34</v>
-      </c>
-      <c r="F23" s="6" t="n">
-        <v>59519.38</v>
+        <v>83551471.34999999</v>
+      </c>
+      <c r="F23" s="8" t="n">
+        <v>55165.31</v>
       </c>
       <c r="G23" s="7" t="n">
-        <v>2318924.87</v>
+        <v>-134373.43</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>2.64</v>
+        <v>-0.16</v>
       </c>
     </row>
     <row r="24">
@@ -2920,22 +2920,22 @@
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>79684306.97</v>
-      </c>
-      <c r="D24" s="6" t="n">
-        <v>52611.99</v>
+        <v>81341602.65000001</v>
+      </c>
+      <c r="D24" s="8" t="n">
+        <v>53706.23</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>80724005.92</v>
-      </c>
-      <c r="F24" s="6" t="n">
-        <v>53298.46</v>
+        <v>81505402.37</v>
+      </c>
+      <c r="F24" s="8" t="n">
+        <v>53814.38</v>
       </c>
       <c r="G24" s="7" t="n">
-        <v>1039698.95</v>
+        <v>163799.72</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>1.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="25">
@@ -2950,22 +2950,22 @@
         </is>
       </c>
       <c r="C25" s="7" t="n">
-        <v>91704370.55</v>
-      </c>
-      <c r="D25" s="6" t="n">
-        <v>60548.3</v>
+        <v>82434422.76000001</v>
+      </c>
+      <c r="D25" s="8" t="n">
+        <v>54427.77</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>93186309.14</v>
-      </c>
-      <c r="F25" s="6" t="n">
-        <v>61526.76</v>
+        <v>81376485.23999999</v>
+      </c>
+      <c r="F25" s="8" t="n">
+        <v>53729.26</v>
       </c>
       <c r="G25" s="7" t="n">
-        <v>1481938.59</v>
+        <v>-1057937.52</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>1.62</v>
+        <v>-1.28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Corregir resultado neto (resultado financiero con signo), flujo de caja sin doble conteo de CT, conciliar ventas/costos con P&L, formato MM/mil M y control de conciliación
</commit_message>
<xml_diff>
--- a/excel/dashboard_costos.xlsx
+++ b/excel/dashboard_costos.xlsx
@@ -392,12 +392,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Costo_Unitario'!$D$2:$D$5</f>
+              <f>'Costo_Unitario'!$D$2:$D$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Costo_Unitario'!$E$2:$E$5</f>
+              <f>'Costo_Unitario'!$E$2:$E$7</f>
             </numRef>
           </val>
         </ser>
@@ -940,7 +940,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>ARS 81,4 M (USD 53,7 k)</t>
+          <t>ARS 88,9 MM (USD 58,7 k)</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>ARS 27,1 M (USD 17,9 k)</t>
+          <t>ARS 27,1 MM (USD 17,9 k)</t>
         </is>
       </c>
     </row>
@@ -964,7 +964,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>ARS 54,3 M (USD 35,9 k)</t>
+          <t>ARS 61,9 MM (USD 40,8 k)</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>25.312</t>
+          <t>61.757</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>-1,28%</t>
+          <t>-1,20%</t>
         </is>
       </c>
     </row>
@@ -1082,19 +1082,19 @@
         <v>14525.62</v>
       </c>
       <c r="E2" s="7" t="n">
-        <v>45447172.45</v>
+        <v>43148868.15</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>30006.74</v>
+        <v>28489.27</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>67447172.45</v>
+        <v>65148868.15</v>
       </c>
       <c r="H2" s="8" t="n">
-        <v>44532.36</v>
+        <v>43014.89</v>
       </c>
       <c r="I2" s="6" t="n">
-        <v>17987</v>
+        <v>67488</v>
       </c>
     </row>
     <row r="3">
@@ -1115,19 +1115,19 @@
         <v>14670.87</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>47179459.18</v>
+        <v>55735514.79</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>31150.49</v>
+        <v>36799.67</v>
       </c>
       <c r="G3" s="7" t="n">
-        <v>69399459.18000001</v>
+        <v>77955514.79000001</v>
       </c>
       <c r="H3" s="8" t="n">
-        <v>45821.37</v>
+        <v>51470.55</v>
       </c>
       <c r="I3" s="6" t="n">
-        <v>18954</v>
+        <v>60995</v>
       </c>
     </row>
     <row r="4">
@@ -1148,19 +1148,19 @@
         <v>14816.13</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>44084639.24</v>
+        <v>50487143.35</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>29107.12</v>
+        <v>33334.41</v>
       </c>
       <c r="G4" s="7" t="n">
-        <v>66524639.24</v>
+        <v>72927143.34999999</v>
       </c>
       <c r="H4" s="8" t="n">
-        <v>43923.25</v>
+        <v>48150.54</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>18289</v>
+        <v>69770</v>
       </c>
     </row>
     <row r="5">
@@ -1181,19 +1181,19 @@
         <v>14961.39</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>44361321.46</v>
+        <v>53695879.59</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>29289.8</v>
+        <v>35452.99</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>67021321.46</v>
+        <v>76355879.59</v>
       </c>
       <c r="H5" s="8" t="n">
-        <v>44251.19</v>
+        <v>50414.38</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>19436</v>
+        <v>68180</v>
       </c>
     </row>
     <row r="6">
@@ -1214,19 +1214,19 @@
         <v>15106.64</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>48186897.22</v>
+        <v>58144310.03</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>31815.66</v>
+        <v>38390.09</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>71066897.22</v>
+        <v>81024310.03</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>46922.3</v>
+        <v>53496.74</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>19158</v>
+        <v>80652</v>
       </c>
     </row>
     <row r="7">
@@ -1247,19 +1247,19 @@
         <v>15251.9</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>49113724.63</v>
+        <v>57621137.52</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>32427.6</v>
+        <v>38044.67</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>72213724.63</v>
+        <v>80721137.52</v>
       </c>
       <c r="H7" s="8" t="n">
-        <v>47679.5</v>
+        <v>53296.56</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>19412</v>
+        <v>62088</v>
       </c>
     </row>
     <row r="8">
@@ -1280,19 +1280,19 @@
         <v>15397.16</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>51165356.46</v>
+        <v>51437228.22</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>33782.2</v>
+        <v>33961.71</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>74485356.45999999</v>
+        <v>74757228.22</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>49179.36</v>
+        <v>49358.86</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>20677</v>
+        <v>64007</v>
       </c>
     </row>
     <row r="9">
@@ -1313,19 +1313,19 @@
         <v>15542.41</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>46201076.56</v>
+        <v>52714226.25</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>30504.51</v>
+        <v>34804.85</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>69741076.56</v>
+        <v>76254226.25</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>46046.92</v>
+        <v>50347.26</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>20899</v>
+        <v>72610</v>
       </c>
     </row>
     <row r="10">
@@ -1346,19 +1346,19 @@
         <v>15687.67</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>44789262.93</v>
+        <v>47993428.46</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>29572.35</v>
+        <v>31687.92</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>68549262.93000001</v>
+        <v>71753428.45999999</v>
       </c>
       <c r="H10" s="8" t="n">
-        <v>45260.02</v>
+        <v>47375.59</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>20199</v>
+        <v>65928</v>
       </c>
     </row>
     <row r="11">
@@ -1379,19 +1379,19 @@
         <v>15832.92</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>46625039.14</v>
+        <v>49956874.03</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>30784.43</v>
+        <v>32984.29</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>70605039.14</v>
+        <v>73936874.03</v>
       </c>
       <c r="H11" s="8" t="n">
-        <v>46617.36</v>
+        <v>48817.22</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>21691</v>
+        <v>53043</v>
       </c>
     </row>
     <row r="12">
@@ -1412,19 +1412,19 @@
         <v>15978.18</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>50478185.96</v>
+        <v>44897318.24</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>33328.49</v>
+        <v>29643.7</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>74678185.95999999</v>
+        <v>69097318.23999999</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>49306.67</v>
+        <v>45621.88</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>22104</v>
+        <v>58951</v>
       </c>
     </row>
     <row r="13">
@@ -1445,19 +1445,19 @@
         <v>16123.44</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>53629693.25</v>
+        <v>45884377.74</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>35409.29</v>
+        <v>30295.41</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>78049693.25</v>
+        <v>70304377.73999999</v>
       </c>
       <c r="H13" s="8" t="n">
-        <v>51532.73</v>
+        <v>46418.84</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>22359</v>
+        <v>58959</v>
       </c>
     </row>
     <row r="14">
@@ -1478,19 +1478,19 @@
         <v>16268.69</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>49535648.68</v>
+        <v>57284377.47</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>32706.18</v>
+        <v>37822.32</v>
       </c>
       <c r="G14" s="7" t="n">
-        <v>74175648.68000001</v>
+        <v>81924377.47</v>
       </c>
       <c r="H14" s="8" t="n">
-        <v>48974.87</v>
+        <v>54091.01</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>21877</v>
+        <v>63324</v>
       </c>
     </row>
     <row r="15">
@@ -1511,19 +1511,19 @@
         <v>16413.95</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>47220987.01</v>
+        <v>66256352.81</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>31177.91</v>
+        <v>43746.11</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>72080987.01000001</v>
+        <v>91116352.81</v>
       </c>
       <c r="H15" s="8" t="n">
-        <v>47591.86</v>
+        <v>60160.06</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>21802</v>
+        <v>66227</v>
       </c>
     </row>
     <row r="16">
@@ -1544,19 +1544,19 @@
         <v>16559.2</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>57291998.11</v>
+        <v>65693380.65</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>37827.35</v>
+        <v>43374.41</v>
       </c>
       <c r="G16" s="7" t="n">
-        <v>82371998.11</v>
+        <v>90773380.65000001</v>
       </c>
       <c r="H16" s="8" t="n">
-        <v>54386.55</v>
+        <v>59933.61</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>23018</v>
+        <v>80731</v>
       </c>
     </row>
     <row r="17">
@@ -1577,19 +1577,19 @@
         <v>16704.46</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>47961981.2</v>
+        <v>76695731.45999999</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>31667.16</v>
+        <v>50638.77</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>73261981.2</v>
+        <v>101995731.46</v>
       </c>
       <c r="H17" s="8" t="n">
-        <v>48371.62</v>
+        <v>67343.23</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>22513</v>
+        <v>69178</v>
       </c>
     </row>
     <row r="18">
@@ -1610,19 +1610,19 @@
         <v>16849.72</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>56355264.81</v>
+        <v>73855523.84</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>37208.87</v>
+        <v>48763.51</v>
       </c>
       <c r="G18" s="7" t="n">
-        <v>81875264.81</v>
+        <v>99375523.84</v>
       </c>
       <c r="H18" s="8" t="n">
-        <v>54058.58</v>
+        <v>65613.22</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>23363</v>
+        <v>64593</v>
       </c>
     </row>
     <row r="19">
@@ -1643,19 +1643,19 @@
         <v>16994.97</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>59399474.56</v>
+        <v>63380673.94</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>39218.82</v>
+        <v>41847.43</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>85139474.56</v>
+        <v>89120673.94</v>
       </c>
       <c r="H19" s="8" t="n">
-        <v>56213.8</v>
+        <v>58842.4</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>24490</v>
+        <v>92129</v>
       </c>
     </row>
     <row r="20">
@@ -1676,19 +1676,19 @@
         <v>17140.23</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>54994124.76</v>
+        <v>66574949.74</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>36310.17</v>
+        <v>43956.47</v>
       </c>
       <c r="G20" s="7" t="n">
-        <v>80954124.76000001</v>
+        <v>92534949.73999999</v>
       </c>
       <c r="H20" s="8" t="n">
-        <v>53450.4</v>
+        <v>61096.7</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>24374</v>
+        <v>80273</v>
       </c>
     </row>
     <row r="21">
@@ -1709,19 +1709,19 @@
         <v>17285.49</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>57352318.33</v>
+        <v>60609124.5</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>37867.18</v>
+        <v>40017.5</v>
       </c>
       <c r="G21" s="7" t="n">
-        <v>83532318.33</v>
+        <v>86789124.5</v>
       </c>
       <c r="H21" s="8" t="n">
-        <v>55152.66</v>
+        <v>57302.99</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>24116</v>
+        <v>67880</v>
       </c>
     </row>
     <row r="22">
@@ -1742,19 +1742,19 @@
         <v>17430.74</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>59498682.88</v>
+        <v>55922492.26</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>39284.32</v>
+        <v>36923.13</v>
       </c>
       <c r="G22" s="7" t="n">
-        <v>85898682.88</v>
+        <v>82322492.26000001</v>
       </c>
       <c r="H22" s="8" t="n">
-        <v>56715.07</v>
+        <v>54353.87</v>
       </c>
       <c r="I22" s="6" t="n">
-        <v>24789</v>
+        <v>67161</v>
       </c>
     </row>
     <row r="23">
@@ -1775,19 +1775,19 @@
         <v>17576</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>56931471.35</v>
+        <v>56506248.32</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>37589.31</v>
+        <v>37308.55</v>
       </c>
       <c r="G23" s="7" t="n">
-        <v>83551471.34999999</v>
+        <v>83126248.31999999</v>
       </c>
       <c r="H23" s="8" t="n">
-        <v>55165.31</v>
+        <v>54884.55</v>
       </c>
       <c r="I23" s="6" t="n">
-        <v>25725</v>
+        <v>66610</v>
       </c>
     </row>
     <row r="24">
@@ -1808,19 +1808,19 @@
         <v>17721.25</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>54665402.37</v>
+        <v>50235389.95</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>36093.13</v>
+        <v>33168.19</v>
       </c>
       <c r="G24" s="7" t="n">
-        <v>81505402.37</v>
+        <v>77075389.95</v>
       </c>
       <c r="H24" s="8" t="n">
-        <v>53814.38</v>
+        <v>50889.44</v>
       </c>
       <c r="I24" s="6" t="n">
-        <v>24959</v>
+        <v>67760</v>
       </c>
     </row>
     <row r="25">
@@ -1841,19 +1841,19 @@
         <v>17866.51</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>54316485.24</v>
+        <v>61866956.82</v>
       </c>
       <c r="F25" s="8" t="n">
-        <v>35862.75</v>
+        <v>40847.99</v>
       </c>
       <c r="G25" s="7" t="n">
-        <v>81376485.23999999</v>
+        <v>88926956.81999999</v>
       </c>
       <c r="H25" s="8" t="n">
-        <v>53729.26</v>
+        <v>58714.5</v>
       </c>
       <c r="I25" s="6" t="n">
-        <v>25312</v>
+        <v>61757</v>
       </c>
     </row>
   </sheetData>
@@ -1925,10 +1925,10 @@
         </is>
       </c>
       <c r="E2" s="7" t="n">
-        <v>34282307.91</v>
+        <v>37716134.42</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>22635.08</v>
+        <v>24902.28</v>
       </c>
     </row>
     <row r="3">
@@ -1953,10 +1953,10 @@
         </is>
       </c>
       <c r="E3" s="7" t="n">
-        <v>22503319.67</v>
+        <v>23615901.07</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>14857.94</v>
+        <v>15592.53</v>
       </c>
     </row>
     <row r="4">
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E4" s="7" t="n">
-        <v>14579868.78</v>
+        <v>16620459.36</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>9626.440000000001</v>
+        <v>10973.75</v>
       </c>
     </row>
     <row r="5">
@@ -2009,10 +2009,10 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>9430632.279999999</v>
+        <v>10974461.97</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>6226.63</v>
+        <v>7245.95</v>
       </c>
     </row>
   </sheetData>
@@ -2027,7 +2027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2066,6 +2066,11 @@
           <t>unidades</t>
         </is>
       </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>costo_ventas_ars</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
@@ -2089,13 +2094,16 @@
         </is>
       </c>
       <c r="E2" s="7" t="n">
-        <v>1397.68</v>
+        <v>1007.33</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>0.92</v>
+        <v>0.67</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>6328</v>
+        <v>10216</v>
+      </c>
+      <c r="H2" s="6" t="n">
+        <v>10290888.49</v>
       </c>
     </row>
     <row r="3">
@@ -2120,13 +2128,16 @@
         </is>
       </c>
       <c r="E3" s="7" t="n">
-        <v>1411.26</v>
+        <v>988.9400000000001</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>0.93</v>
+        <v>0.65</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>6328</v>
+        <v>9116</v>
+      </c>
+      <c r="H3" s="6" t="n">
+        <v>9015188.810000001</v>
       </c>
     </row>
     <row r="4">
@@ -2151,13 +2162,16 @@
         </is>
       </c>
       <c r="E4" s="7" t="n">
-        <v>2068.76</v>
+        <v>1099.3</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>1.37</v>
+        <v>0.73</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>6328</v>
+        <v>14010</v>
+      </c>
+      <c r="H4" s="6" t="n">
+        <v>15401139.88</v>
       </c>
     </row>
     <row r="5">
@@ -2182,13 +2196,84 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>1700.94</v>
+        <v>1016.11</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>1.12</v>
+        <v>0.67</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>6328</v>
+        <v>8940</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>9083996.57</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NovaCampo Alimentos S.A.</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>NC-005</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Dulce de leche 450g</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>1022.62</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>10163</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>10392920.42</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>NovaCampo Alimentos S.A.</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>NC-006</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Galletitas surtidas 300g</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>952.11</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>9312</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>8866054.539999999</v>
       </c>
     </row>
   </sheetData>
@@ -2260,22 +2345,22 @@
         </is>
       </c>
       <c r="C2" s="7" t="n">
-        <v>64782056.64</v>
+        <v>63540968.19</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>42772.7</v>
+        <v>41953.27</v>
       </c>
       <c r="E2" s="7" t="n">
-        <v>67447172.45</v>
+        <v>65148868.15</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>44532.36</v>
+        <v>43014.89</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>2665115.8</v>
+        <v>1607899.96</v>
       </c>
       <c r="H2" s="6" t="n">
-        <v>4.11</v>
+        <v>2.53</v>
       </c>
     </row>
     <row r="3">
@@ -2290,22 +2375,22 @@
         </is>
       </c>
       <c r="C3" s="7" t="n">
-        <v>67535408.61</v>
+        <v>76007086.34999999</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>44590.62</v>
+        <v>50184.09</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>69399459.18000001</v>
+        <v>77955514.79000001</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>45821.37</v>
+        <v>51470.55</v>
       </c>
       <c r="G3" s="7" t="n">
-        <v>1864050.57</v>
+        <v>1948428.44</v>
       </c>
       <c r="H3" s="6" t="n">
-        <v>2.76</v>
+        <v>2.56</v>
       </c>
     </row>
     <row r="4">
@@ -2320,22 +2405,22 @@
         </is>
       </c>
       <c r="C4" s="7" t="n">
-        <v>65623189.89</v>
+        <v>72890226.81999999</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>43328.06</v>
+        <v>48126.16</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>66524639.24</v>
+        <v>72927143.34999999</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>43923.25</v>
+        <v>48150.54</v>
       </c>
       <c r="G4" s="7" t="n">
-        <v>901449.35</v>
+        <v>36916.53</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>1.37</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="5">
@@ -2350,22 +2435,22 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>66358325.49</v>
+        <v>76082823.31999999</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>43813.44</v>
+        <v>50234.09</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>67021321.46</v>
+        <v>76355879.59</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>44251.19</v>
+        <v>50414.38</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>662995.97</v>
+        <v>273056.27</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>1</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="6">
@@ -2380,22 +2465,22 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>68824411.19</v>
+        <v>79285202.05</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>45441.69</v>
+        <v>52348.48</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>71066897.22</v>
+        <v>81024310.03</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>46922.3</v>
+        <v>53496.74</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>2242486.03</v>
+        <v>1739107.98</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>3.26</v>
+        <v>2.19</v>
       </c>
     </row>
     <row r="7">
@@ -2410,22 +2495,22 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>71295683.23</v>
+        <v>80063352.47</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>47073.36</v>
+        <v>52862.26</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>72213724.63</v>
+        <v>80721137.52</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>47679.5</v>
+        <v>53296.56</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>918041.41</v>
+        <v>657785.05</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>1.29</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="8">
@@ -2440,22 +2525,22 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>72971842.09</v>
+        <v>72398295.34999999</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>48180.05</v>
+        <v>47801.36</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>74485356.45999999</v>
+        <v>74757228.22</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>49179.36</v>
+        <v>49358.86</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>1513514.37</v>
+        <v>2358932.87</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>2.07</v>
+        <v>3.26</v>
       </c>
     </row>
     <row r="9">
@@ -2470,22 +2555,22 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>69012803.77</v>
+        <v>75284818.59999999</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>45566.07</v>
+        <v>49707.21</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>69741076.56</v>
+        <v>76254226.25</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>46046.92</v>
+        <v>50347.26</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>728272.79</v>
+        <v>969407.65</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>1.06</v>
+        <v>1.29</v>
       </c>
     </row>
     <row r="10">
@@ -2500,22 +2585,22 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>69448960.15000001</v>
+        <v>72823656.28</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>45854.05</v>
+        <v>48082.21</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>68549262.93000001</v>
+        <v>71753428.45999999</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>45260.02</v>
+        <v>47375.59</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>-899697.22</v>
+        <v>-1070227.82</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>-1.3</v>
+        <v>-1.47</v>
       </c>
     </row>
     <row r="11">
@@ -2530,22 +2615,22 @@
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>68201733.8</v>
+        <v>71410563.42</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>45030.56</v>
+        <v>47149.21</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>70605039.14</v>
+        <v>73936874.03</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>46617.36</v>
+        <v>48817.22</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>2403305.34</v>
+        <v>2526310.61</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>3.52</v>
+        <v>3.54</v>
       </c>
     </row>
     <row r="12">
@@ -2560,22 +2645,22 @@
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>72641439.17</v>
+        <v>66743953.27</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>47961.9</v>
+        <v>44068.05</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>74678185.95999999</v>
+        <v>69097318.23999999</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>49306.67</v>
+        <v>45621.88</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>2036746.79</v>
+        <v>2353364.97</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>2.8</v>
+        <v>3.53</v>
       </c>
     </row>
     <row r="13">
@@ -2590,22 +2675,22 @@
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>75939001.73</v>
+        <v>69788902.65000001</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>50139.13</v>
+        <v>46078.5</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>78049693.25</v>
+        <v>70304377.73999999</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>51532.73</v>
+        <v>46418.84</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>2110691.52</v>
+        <v>515475.09</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>2.78</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="14">
@@ -2620,22 +2705,22 @@
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>74150685.5</v>
+        <v>78752384.14</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>48958.39</v>
+        <v>51996.68</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>74175648.68000001</v>
+        <v>81924377.47</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>48974.87</v>
+        <v>54091.01</v>
       </c>
       <c r="G14" s="7" t="n">
-        <v>24963.18</v>
+        <v>3171993.33</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>0.03</v>
+        <v>4.03</v>
       </c>
     </row>
     <row r="15">
@@ -2650,22 +2735,22 @@
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>69472627.09</v>
+        <v>88278374.62</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>45869.67</v>
+        <v>58286.27</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>72080987.01000001</v>
+        <v>91116352.81</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>47591.86</v>
+        <v>60160.06</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>2608359.91</v>
+        <v>2837978.19</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>3.75</v>
+        <v>3.21</v>
       </c>
     </row>
     <row r="16">
@@ -2680,22 +2765,22 @@
         </is>
       </c>
       <c r="C16" s="7" t="n">
-        <v>81340910.84999999</v>
+        <v>91445020.14</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>53705.77</v>
+        <v>60377.07</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>82371998.11</v>
+        <v>90773380.65000001</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>54386.55</v>
+        <v>59933.61</v>
       </c>
       <c r="G16" s="7" t="n">
-        <v>1031087.26</v>
+        <v>-671639.49</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>1.27</v>
+        <v>-0.73</v>
       </c>
     </row>
     <row r="17">
@@ -2710,22 +2795,22 @@
         </is>
       </c>
       <c r="C17" s="7" t="n">
-        <v>70620222.58</v>
+        <v>98583284.81</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>46627.38</v>
+        <v>65090.14</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>73261981.2</v>
+        <v>101995731.46</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>48371.62</v>
+        <v>67343.23</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>2641758.62</v>
+        <v>3412446.65</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>3.74</v>
+        <v>3.46</v>
       </c>
     </row>
     <row r="18">
@@ -2740,22 +2825,22 @@
         </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>79162315.17</v>
+        <v>97795158.39</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>52267.34</v>
+        <v>64569.78</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>81875264.81</v>
+        <v>99375523.84</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>54058.58</v>
+        <v>65613.22</v>
       </c>
       <c r="G18" s="7" t="n">
-        <v>2712949.64</v>
+        <v>1580365.45</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>3.43</v>
+        <v>1.62</v>
       </c>
     </row>
     <row r="19">
@@ -2770,22 +2855,22 @@
         </is>
       </c>
       <c r="C19" s="7" t="n">
-        <v>82219629.08</v>
+        <v>87294691.73</v>
       </c>
       <c r="D19" s="8" t="n">
-        <v>54285.95</v>
+        <v>57636.79</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>85139474.56</v>
+        <v>89120673.94</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>56213.8</v>
+        <v>58842.4</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>2919845.48</v>
+        <v>1825982.21</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>3.55</v>
+        <v>2.09</v>
       </c>
     </row>
     <row r="20">
@@ -2800,22 +2885,22 @@
         </is>
       </c>
       <c r="C20" s="7" t="n">
-        <v>79525997.79000001</v>
+        <v>90027380.67</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>52507.47</v>
+        <v>59441.06</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>80954124.76000001</v>
+        <v>92534949.73999999</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>53450.4</v>
+        <v>61096.7</v>
       </c>
       <c r="G20" s="7" t="n">
-        <v>1428126.97</v>
+        <v>2507569.07</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>1.8</v>
+        <v>2.79</v>
       </c>
     </row>
     <row r="21">
@@ -2830,22 +2915,22 @@
         </is>
       </c>
       <c r="C21" s="7" t="n">
-        <v>83804937.81</v>
+        <v>88123863.31</v>
       </c>
       <c r="D21" s="8" t="n">
-        <v>55332.66</v>
+        <v>58184.25</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>83532318.33</v>
+        <v>86789124.5</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>55152.66</v>
+        <v>57302.99</v>
       </c>
       <c r="G21" s="7" t="n">
-        <v>-272619.48</v>
+        <v>-1334738.81</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-0.33</v>
+        <v>-1.51</v>
       </c>
     </row>
     <row r="22">
@@ -2860,22 +2945,22 @@
         </is>
       </c>
       <c r="C22" s="7" t="n">
-        <v>86393144.72</v>
+        <v>79633335.61</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>57041.54</v>
+        <v>52578.34</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>85898682.88</v>
+        <v>82322492.26000001</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>56715.07</v>
+        <v>54353.87</v>
       </c>
       <c r="G22" s="7" t="n">
-        <v>-494461.85</v>
+        <v>2689156.65</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>-0.57</v>
+        <v>3.38</v>
       </c>
     </row>
     <row r="23">
@@ -2890,22 +2975,22 @@
         </is>
       </c>
       <c r="C23" s="7" t="n">
-        <v>83685844.78</v>
+        <v>83076719.89</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>55254.03</v>
+        <v>54851.85</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>83551471.34999999</v>
+        <v>83126248.31999999</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>55165.31</v>
+        <v>54884.55</v>
       </c>
       <c r="G23" s="7" t="n">
-        <v>-134373.43</v>
+        <v>49528.43</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>-0.16</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="24">
@@ -2920,22 +3005,22 @@
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>81341602.65000001</v>
+        <v>76829858.34</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>53706.23</v>
+        <v>50727.33</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>81505402.37</v>
+        <v>77075389.95</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>53814.38</v>
+        <v>50889.44</v>
       </c>
       <c r="G24" s="7" t="n">
-        <v>163799.72</v>
+        <v>245531.61</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>0.2</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="25">
@@ -2950,22 +3035,22 @@
         </is>
       </c>
       <c r="C25" s="7" t="n">
-        <v>82434422.76000001</v>
+        <v>90011133.15000001</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>54427.77</v>
+        <v>59430.33</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>81376485.23999999</v>
+        <v>88926956.81999999</v>
       </c>
       <c r="F25" s="8" t="n">
-        <v>53729.26</v>
+        <v>58714.5</v>
       </c>
       <c r="G25" s="7" t="n">
-        <v>-1057937.52</v>
+        <v>-1084176.33</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-1.28</v>
+        <v>-1.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>